<commit_message>
fix: untuk list di project overview belum rapih [2026-06-23 16:28]
</commit_message>
<xml_diff>
--- a/projects.xlsx
+++ b/projects.xlsx
@@ -960,7 +960,7 @@
       </c>
       <c r="I4" s="23" t="inlineStr">
         <is>
-          <t>January 2026</t>
+          <t>January 2026 - May 2026</t>
         </is>
       </c>
       <c r="J4" s="23" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="I5" s="24" t="inlineStr">
         <is>
-          <t>August 2025</t>
+          <t>August 2025 - March 2026</t>
         </is>
       </c>
       <c r="J5" s="24" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="I6" s="25" t="inlineStr">
         <is>
-          <t>May 2025</t>
+          <t>May 2025 - May 2025</t>
         </is>
       </c>
       <c r="J6" s="25" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="I7" s="24" t="inlineStr">
         <is>
-          <t>March 2025</t>
+          <t>March 2025 - March 2025</t>
         </is>
       </c>
       <c r="J7" s="24" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="I8" s="25" t="inlineStr">
         <is>
-          <t>February 2025</t>
+          <t>February 2025 - May 2025</t>
         </is>
       </c>
       <c r="J8" s="25" t="inlineStr">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="I9" s="24" t="inlineStr">
         <is>
-          <t>January 2025</t>
+          <t>January 2025 - April 2025</t>
         </is>
       </c>
       <c r="J9" s="24" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="I10" s="25" t="inlineStr">
         <is>
-          <t>September 2024</t>
+          <t>September 2024 - November 2024</t>
         </is>
       </c>
       <c r="J10" s="25" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="I11" s="24" t="inlineStr">
         <is>
-          <t>July 2024</t>
+          <t>July 2024 - August 2024</t>
         </is>
       </c>
       <c r="J11" s="24" t="inlineStr">

</xml_diff>